<commit_message>
Rebuild Alphabet memo for PM readiness
</commit_message>
<xml_diff>
--- a/nvidia/model.xlsx
+++ b/nvidia/model.xlsx
@@ -100,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,7 +127,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -2431,7 +2430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2575,138 +2574,54 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Risk / reward</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="n">
-        <v>0.006457311149012426</v>
+          <t>Scenario expected value</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>224.9106059379768</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>long framing</t>
+          <t>illustrative probability-weighted arithmetic</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Payoff ratio b</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Position size</t>
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>0.006457311149012426</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>reward / risk</t>
+          <t>no capital recommendation</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>p(win)</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="n">
-        <v>0.75</v>
+          <t>Binding constraint</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>implementation evidence missing</t>
+        </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>probability mass favouring the position</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Kelly f</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>-37.96580511312897</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>implementation inputs missing</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Quarter-Kelly</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>0.25 x Kelly</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Liquidity cap</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="n">
-        <v>27.29</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>20% of ADV over 5 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Risk-budget cap</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>0.02145928366240926</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>1.5% of NAV at risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Concentration cap</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>single-name hard limit</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Position size</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>binding: quarter-Kelly</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Basis: illustrative $1bn book. Illustrative only.</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Basis: no capital recommendation; implementation inputs missing. Illustrative only.</t>
         </is>
       </c>
     </row>
@@ -2735,90 +2650,90 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Base year: trailing twelve months to 2026-04-26, all statement inputs from SEC XBRL companyconcept (CIK 0001045810).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Quarterly series are reconstructed from filed facts: Q4 is derived as fiscal year minus the nine-month cumulative, and cash-flow items are unwound from year-to-date cumulatives.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Consensus estimates and price targets: FMP analyst/financial-estimates and analyst/price-target-consensus, retrieved 2026-08-07.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Segment revenue: FMP statements/revenue-product-segmentation. No SEC fallback exists because companyfacts flattens dimensioned facts; the segment sum is reconciled to consolidated revenue.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr"/>
+      <c r="A7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>YEAR-1 CAPEX ANCHOR. No capex guidance is published for this filer, so year 1 is $1.8bn reported plus 3 quarter(s) at the $1.8bn exit rate, giving $7.0bn.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr"/>
+      <c r="A9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>YEAR-1 SEGMENT ANCHOR. No quarterly segment actuals are recorded for this filer, so year-1 segment revenue is checked only at the consolidated level.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="inlineStr"/>
+      <c r="A11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>DISCOUNT RATE. WACC is an input cell on Drivers and every discounted line references it, so changing it here re-values the model. It is worth knowing what that is worth: terminal value is 71% of enterprise value, the base case discounts at 9.75% giving $197.39, published third-party WACC estimates cluster near 7.57% giving $290.14, and the reverse DCF implies the market is discounting at 8.94%. The discount rate moves this valuation more than the depreciation schedule does.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr"/>
+      <c r="A13" s="23" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>MODEL DESIGN. We forecast EBITDA margin and derive EBIT by subtracting a depreciation schedule built from capex vintages. Forecasting EBIT margin directly hides the depreciation assumption.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr"/>
+      <c r="A15" s="23" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>KEY LIMITATION. The asset-life split driving the depreciation schedule is a stated assumption calibrated to reported D&amp;A, not a disclosed figure. It is the most load-bearing assumption in the model.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="24" t="inlineStr"/>
+      <c r="A17" s="23" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="24" t="inlineStr">
-        <is>
-          <t>This is analytical research on public information. Not investment advice, not a recommendation to any person, and not a solicitation. Position sizing is illustrative against a notional $1bn book.</t>
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>This is analytical research on public information. Not investment advice, not a recommendation to any person, and not a solicitation. No percentage sizing is provided without implementation and portfolio inputs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild Alphabet memo for PM readiness (#8)
</commit_message>
<xml_diff>
--- a/nvidia/model.xlsx
+++ b/nvidia/model.xlsx
@@ -100,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,7 +127,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -2431,7 +2430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2575,138 +2574,54 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Risk / reward</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="n">
-        <v>0.006457311149012426</v>
+          <t>Scenario expected value</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>224.9106059379768</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>long framing</t>
+          <t>illustrative probability-weighted arithmetic</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Payoff ratio b</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Position size</t>
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>0.006457311149012426</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>reward / risk</t>
+          <t>no capital recommendation</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>p(win)</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="n">
-        <v>0.75</v>
+          <t>Binding constraint</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>implementation evidence missing</t>
+        </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>probability mass favouring the position</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Kelly f</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>-37.96580511312897</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>implementation inputs missing</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Quarter-Kelly</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>0.25 x Kelly</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Liquidity cap</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="n">
-        <v>27.29</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>20% of ADV over 5 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Risk-budget cap</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>0.02145928366240926</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>1.5% of NAV at risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Concentration cap</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>single-name hard limit</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Position size</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>binding: quarter-Kelly</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Basis: illustrative $1bn book. Illustrative only.</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Basis: no capital recommendation; implementation inputs missing. Illustrative only.</t>
         </is>
       </c>
     </row>
@@ -2735,90 +2650,90 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Base year: trailing twelve months to 2026-04-26, all statement inputs from SEC XBRL companyconcept (CIK 0001045810).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Quarterly series are reconstructed from filed facts: Q4 is derived as fiscal year minus the nine-month cumulative, and cash-flow items are unwound from year-to-date cumulatives.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Consensus estimates and price targets: FMP analyst/financial-estimates and analyst/price-target-consensus, retrieved 2026-08-07.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Segment revenue: FMP statements/revenue-product-segmentation. No SEC fallback exists because companyfacts flattens dimensioned facts; the segment sum is reconciled to consolidated revenue.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr"/>
+      <c r="A7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>YEAR-1 CAPEX ANCHOR. No capex guidance is published for this filer, so year 1 is $1.8bn reported plus 3 quarter(s) at the $1.8bn exit rate, giving $7.0bn.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr"/>
+      <c r="A9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>YEAR-1 SEGMENT ANCHOR. No quarterly segment actuals are recorded for this filer, so year-1 segment revenue is checked only at the consolidated level.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="inlineStr"/>
+      <c r="A11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>DISCOUNT RATE. WACC is an input cell on Drivers and every discounted line references it, so changing it here re-values the model. It is worth knowing what that is worth: terminal value is 71% of enterprise value, the base case discounts at 9.75% giving $197.39, published third-party WACC estimates cluster near 7.57% giving $290.14, and the reverse DCF implies the market is discounting at 8.94%. The discount rate moves this valuation more than the depreciation schedule does.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr"/>
+      <c r="A13" s="23" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>MODEL DESIGN. We forecast EBITDA margin and derive EBIT by subtracting a depreciation schedule built from capex vintages. Forecasting EBIT margin directly hides the depreciation assumption.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr"/>
+      <c r="A15" s="23" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>KEY LIMITATION. The asset-life split driving the depreciation schedule is a stated assumption calibrated to reported D&amp;A, not a disclosed figure. It is the most load-bearing assumption in the model.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="24" t="inlineStr"/>
+      <c r="A17" s="23" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="24" t="inlineStr">
-        <is>
-          <t>This is analytical research on public information. Not investment advice, not a recommendation to any person, and not a solicitation. Position sizing is illustrative against a notional $1bn book.</t>
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>This is analytical research on public information. Not investment advice, not a recommendation to any person, and not a solicitation. No percentage sizing is provided without implementation and portfolio inputs.</t>
         </is>
       </c>
     </row>

</xml_diff>